<commit_message>
Remove medium badge from cards, add assigned person field on card creation and detail edit
</commit_message>
<xml_diff>
--- a/data/task-management.xlsx
+++ b/data/task-management.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="186">
   <si>
     <t>UserID</t>
   </si>
@@ -135,6 +135,33 @@
     <t>2026-09-04T07:23:25.120Z</t>
   </si>
   <si>
+    <t>BOARD-dd8d8Y0D</t>
+  </si>
+  <si>
+    <t>OWASP Updates</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:16:56.748Z</t>
+  </si>
+  <si>
+    <t>BOARD-GPtUcHDT</t>
+  </si>
+  <si>
+    <t>NextGen</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:13.224Z</t>
+  </si>
+  <si>
+    <t>BOARD-YCkJVtYj</t>
+  </si>
+  <si>
+    <t>Bugathon Updates</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:21.417Z</t>
+  </si>
+  <si>
     <t>ListID</t>
   </si>
   <si>
@@ -189,6 +216,72 @@
     <t>Status</t>
   </si>
   <si>
+    <t>CARD-rkDBNuM4</t>
+  </si>
+  <si>
+    <t>Logo</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:42.723Z</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:21:02.912Z</t>
+  </si>
+  <si>
+    <t>COMPLETED</t>
+  </si>
+  <si>
+    <t>CARD-8qeH-06h</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:46.492Z</t>
+  </si>
+  <si>
+    <t>TODO</t>
+  </si>
+  <si>
+    <t>CARD-qoYMpst5</t>
+  </si>
+  <si>
+    <t>Agenda</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:55.127Z</t>
+  </si>
+  <si>
+    <t>CARD-fCoghZlP</t>
+  </si>
+  <si>
+    <t>Hall Of Fame</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:59.720Z</t>
+  </si>
+  <si>
+    <t>CARD-FIT2AkSf</t>
+  </si>
+  <si>
+    <t>Skill Bridge</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:18:04.669Z</t>
+  </si>
+  <si>
+    <t>CARD-_K0t2WZj</t>
+  </si>
+  <si>
+    <t>SDEP (Student Developer Expo Prog)</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:18:25.138Z</t>
+  </si>
+  <si>
     <t>UpdateID</t>
   </si>
   <si>
@@ -201,6 +294,24 @@
     <t>Progress</t>
   </si>
   <si>
+    <t>UPD-CYw0R8O_</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>asdasd</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:21:01.458Z</t>
+  </si>
+  <si>
+    <t>UPD-7a2_iMz3</t>
+  </si>
+  <si>
+    <t>asdfsdaf</t>
+  </si>
+  <si>
     <t>ActivityID</t>
   </si>
   <si>
@@ -225,9 +336,6 @@
     <t>Created card</t>
   </si>
   <si>
-    <t>Logo</t>
-  </si>
-  <si>
     <t>2026-09-04T07:23:53.517Z</t>
   </si>
   <si>
@@ -237,9 +345,6 @@
     <t>CARD-y75Q3FLy</t>
   </si>
   <si>
-    <t>Magazine</t>
-  </si>
-  <si>
     <t>2026-09-04T07:24:02.126Z</t>
   </si>
   <si>
@@ -258,9 +363,6 @@
     <t>Changed status</t>
   </si>
   <si>
-    <t>TODO</t>
-  </si>
-  <si>
     <t>IN PROGRESS</t>
   </si>
   <si>
@@ -270,9 +372,6 @@
     <t>ACT-zW2LshVp</t>
   </si>
   <si>
-    <t>COMPLETED</t>
-  </si>
-  <si>
     <t>2026-09-04T07:32:05.903Z</t>
   </si>
   <si>
@@ -376,6 +475,105 @@
   </si>
   <si>
     <t>2026-09-04T08:05:23.431Z</t>
+  </si>
+  <si>
+    <t>ACT-Qb14nG3j</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:42.735Z</t>
+  </si>
+  <si>
+    <t>ACT-YInSpchP</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:46.512Z</t>
+  </si>
+  <si>
+    <t>ACT-BWJb7AzV</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:55.144Z</t>
+  </si>
+  <si>
+    <t>ACT-vrv7YSWn</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:59.733Z</t>
+  </si>
+  <si>
+    <t>ACT--rsNS8i-</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:18:04.684Z</t>
+  </si>
+  <si>
+    <t>ACT-Np04NN4h</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:18:25.150Z</t>
+  </si>
+  <si>
+    <t>ACT-964JIQcv</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:50.217Z</t>
+  </si>
+  <si>
+    <t>ACT-Vh0Hsf8B</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:50.273Z</t>
+  </si>
+  <si>
+    <t>ACT-TzKXHnH7</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:51.206Z</t>
+  </si>
+  <si>
+    <t>ACT-6aMS9zA6</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:51.252Z</t>
+  </si>
+  <si>
+    <t>ACT-nnA4TeDp</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:52.149Z</t>
+  </si>
+  <si>
+    <t>ACT-gBp0x7LM</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:52.200Z</t>
+  </si>
+  <si>
+    <t>ACT-vIycTKBg</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:52.989Z</t>
+  </si>
+  <si>
+    <t>ACT-WbIKGDta</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:20:53.032Z</t>
+  </si>
+  <si>
+    <t>ACT-51wc8kUf</t>
+  </si>
+  <si>
+    <t>Added daily update</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:21:01.475Z</t>
+  </si>
+  <si>
+    <t>ACT-62UjojKV</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:21:02.925Z</t>
   </si>
 </sst>
 </file>
@@ -895,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="15" customWidth="1"/>
@@ -944,6 +1142,75 @@
         <v>38</v>
       </c>
       <c r="G2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -963,16 +1230,16 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>6</v>
@@ -980,53 +1247,53 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
         <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
         <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1037,7 +1304,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="13" width="15" customWidth="1"/>
@@ -1045,31 +1312,31 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>32</v>
@@ -1081,7 +1348,253 @@
         <v>33</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L2" t="s">
+        <v>70</v>
+      </c>
+      <c r="M2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L3" t="s">
+        <v>74</v>
+      </c>
+      <c r="M3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K4" t="s">
+        <v>78</v>
+      </c>
+      <c r="L4" t="s">
+        <v>78</v>
+      </c>
+      <c r="M4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>68</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" t="s">
+        <v>81</v>
+      </c>
+      <c r="M5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+      <c r="J6" t="s">
+        <v>7</v>
+      </c>
+      <c r="K6" t="s">
+        <v>84</v>
+      </c>
+      <c r="L6" t="s">
+        <v>84</v>
+      </c>
+      <c r="M6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
+      <c r="J7" t="s">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>87</v>
+      </c>
+      <c r="L7" t="s">
+        <v>87</v>
+      </c>
+      <c r="M7" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1092,7 +1605,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="9" width="15" customWidth="1"/>
@@ -1100,31 +1613,89 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2">
+        <v>100</v>
+      </c>
+      <c r="H2" t="s">
+        <v>95</v>
+      </c>
+      <c r="I2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3">
+        <v>100</v>
+      </c>
+      <c r="H3" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1135,7 +1706,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="15" customWidth="1"/>
@@ -1143,62 +1714,62 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" t="s">
         <v>67</v>
       </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" t="s">
-        <v>69</v>
-      </c>
       <c r="G2" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>105</v>
       </c>
       <c r="E3" t="s">
         <v>37</v>
@@ -1207,467 +1778,835 @@
         <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>74</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E4" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="G5" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E6" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F6" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="G6" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G7" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="G8" t="s">
-        <v>89</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E9" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="G9" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E10" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G10" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
         <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E11" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="F11" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="G11" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E12" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="G12" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C13" t="s">
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="G13" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C14" t="s">
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E14" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G14" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
         <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="F15" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="G15" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>137</v>
+      </c>
+      <c r="B16" t="s">
         <v>104</v>
       </c>
-      <c r="B16" t="s">
-        <v>67</v>
-      </c>
       <c r="C16" t="s">
         <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E16" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="F16" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="G16" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C17" t="s">
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="F17" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="G17" t="s">
-        <v>107</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>108</v>
+        <v>141</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
       </c>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E18" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F18" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G18" t="s">
-        <v>109</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C19" t="s">
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E19" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="F19" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="G19" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C20" t="s">
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E20" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F20" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="G20" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>147</v>
+      </c>
+      <c r="B21" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" t="s">
         <v>114</v>
       </c>
-      <c r="B21" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" t="s">
-        <v>79</v>
-      </c>
       <c r="E21" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="G21" t="s">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C22" t="s">
         <v>7</v>
       </c>
       <c r="D22" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E22" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="F22" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="G22" t="s">
-        <v>117</v>
+        <v>150</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>118</v>
+        <v>151</v>
       </c>
       <c r="B23" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" t="s">
+        <v>115</v>
+      </c>
+      <c r="F23" t="s">
+        <v>71</v>
+      </c>
+      <c r="G23" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>153</v>
+      </c>
+      <c r="B24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" t="s">
+        <v>105</v>
+      </c>
+      <c r="E24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" t="s">
         <v>67</v>
       </c>
-      <c r="C23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="G24" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>155</v>
+      </c>
+      <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" t="s">
+        <v>105</v>
+      </c>
+      <c r="E25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" t="s">
+        <v>73</v>
+      </c>
+      <c r="G25" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>157</v>
+      </c>
+      <c r="B26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" t="s">
+        <v>77</v>
+      </c>
+      <c r="G26" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>159</v>
+      </c>
+      <c r="B27" t="s">
         <v>79</v>
       </c>
-      <c r="E23" t="s">
-        <v>81</v>
-      </c>
-      <c r="F23" t="s">
-        <v>84</v>
-      </c>
-      <c r="G23" t="s">
-        <v>119</v>
+      <c r="C27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>105</v>
+      </c>
+      <c r="E27" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" t="s">
+        <v>80</v>
+      </c>
+      <c r="G27" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>161</v>
+      </c>
+      <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" t="s">
+        <v>83</v>
+      </c>
+      <c r="G28" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" t="s">
+        <v>105</v>
+      </c>
+      <c r="E29" t="s">
+        <v>37</v>
+      </c>
+      <c r="F29" t="s">
+        <v>86</v>
+      </c>
+      <c r="G29" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>165</v>
+      </c>
+      <c r="B30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" t="s">
+        <v>111</v>
+      </c>
+      <c r="E30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F30" t="s">
+        <v>54</v>
+      </c>
+      <c r="G30" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>167</v>
+      </c>
+      <c r="B31" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" t="s">
+        <v>114</v>
+      </c>
+      <c r="E31" t="s">
+        <v>75</v>
+      </c>
+      <c r="F31" t="s">
+        <v>115</v>
+      </c>
+      <c r="G31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" t="s">
+        <v>111</v>
+      </c>
+      <c r="E32" t="s">
+        <v>54</v>
+      </c>
+      <c r="F32" t="s">
+        <v>57</v>
+      </c>
+      <c r="G32" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>171</v>
+      </c>
+      <c r="B33" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" t="s">
+        <v>114</v>
+      </c>
+      <c r="E33" t="s">
+        <v>115</v>
+      </c>
+      <c r="F33" t="s">
+        <v>71</v>
+      </c>
+      <c r="G33" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>173</v>
+      </c>
+      <c r="B34" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" t="s">
+        <v>111</v>
+      </c>
+      <c r="E34" t="s">
+        <v>57</v>
+      </c>
+      <c r="F34" t="s">
+        <v>54</v>
+      </c>
+      <c r="G34" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>175</v>
+      </c>
+      <c r="B35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C35" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" t="s">
+        <v>114</v>
+      </c>
+      <c r="E35" t="s">
+        <v>71</v>
+      </c>
+      <c r="F35" t="s">
+        <v>115</v>
+      </c>
+      <c r="G35" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>177</v>
+      </c>
+      <c r="B36" t="s">
+        <v>66</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" t="s">
+        <v>54</v>
+      </c>
+      <c r="F36" t="s">
+        <v>51</v>
+      </c>
+      <c r="G36" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>179</v>
+      </c>
+      <c r="B37" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" t="s">
+        <v>114</v>
+      </c>
+      <c r="E37" t="s">
+        <v>115</v>
+      </c>
+      <c r="F37" t="s">
+        <v>71</v>
+      </c>
+      <c r="G37" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>181</v>
+      </c>
+      <c r="B38" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" t="s">
+        <v>182</v>
+      </c>
+      <c r="E38" t="s">
+        <v>37</v>
+      </c>
+      <c r="F38" t="s">
+        <v>94</v>
+      </c>
+      <c r="G38" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" t="s">
+        <v>182</v>
+      </c>
+      <c r="E39" t="s">
+        <v>37</v>
+      </c>
+      <c r="F39" t="s">
+        <v>97</v>
+      </c>
+      <c r="G39" t="s">
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Display priority badge on cards, prompt for priority on creation, and auto-sort lists by priority
</commit_message>
<xml_diff>
--- a/data/task-management.xlsx
+++ b/data/task-management.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="194">
   <si>
     <t>UserID</t>
   </si>
@@ -216,34 +216,250 @@
     <t>Status</t>
   </si>
   <si>
+    <t>CARD-aO6sd2D-</t>
+  </si>
+  <si>
+    <t>Logo</t>
+  </si>
+  <si>
+    <t>Ashik</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:23:31.578Z</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:23:35.112Z</t>
+  </si>
+  <si>
+    <t>COMPLETED</t>
+  </si>
+  <si>
+    <t>UpdateID</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>UpdateText</t>
+  </si>
+  <si>
+    <t>Progress</t>
+  </si>
+  <si>
+    <t>UPD-CYw0R8O_</t>
+  </si>
+  <si>
     <t>CARD-rkDBNuM4</t>
   </si>
   <si>
-    <t>Logo</t>
-  </si>
-  <si>
-    <t>MEDIUM</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:17:42.723Z</t>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>asdasd</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:21:01.458Z</t>
+  </si>
+  <si>
+    <t>UPD-7a2_iMz3</t>
+  </si>
+  <si>
+    <t>asdfsdaf</t>
   </si>
   <si>
     <t>2026-09-04T08:21:02.912Z</t>
   </si>
   <si>
-    <t>COMPLETED</t>
+    <t>ActivityID</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>OldValue</t>
+  </si>
+  <si>
+    <t>NewValue</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>ACT-QCKcrs0o</t>
+  </si>
+  <si>
+    <t>CARD-wiVR66sH</t>
+  </si>
+  <si>
+    <t>Created card</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:23:53.517Z</t>
+  </si>
+  <si>
+    <t>ACT-6S9gKyUQ</t>
+  </si>
+  <si>
+    <t>CARD-y75Q3FLy</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:24:02.126Z</t>
+  </si>
+  <si>
+    <t>ACT-8Z7tZiIR</t>
+  </si>
+  <si>
+    <t>Moved card</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:04.946Z</t>
+  </si>
+  <si>
+    <t>ACT-unq1XO_V</t>
+  </si>
+  <si>
+    <t>Changed status</t>
+  </si>
+  <si>
+    <t>TODO</t>
+  </si>
+  <si>
+    <t>IN PROGRESS</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:05.842Z</t>
+  </si>
+  <si>
+    <t>ACT-zW2LshVp</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:05.903Z</t>
+  </si>
+  <si>
+    <t>ACT-G9JlU1GN</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:07.836Z</t>
+  </si>
+  <si>
+    <t>ACT-hP5mkb6C</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:15.843Z</t>
+  </si>
+  <si>
+    <t>ACT-yZk50wkS</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:15.910Z</t>
+  </si>
+  <si>
+    <t>ACT-kxPkqAQN</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:25.500Z</t>
+  </si>
+  <si>
+    <t>ACT-Nlwsh-Nr</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:25.561Z</t>
+  </si>
+  <si>
+    <t>ACT-IszKmJ30</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:27.279Z</t>
+  </si>
+  <si>
+    <t>ACT-egJr9HT1</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:27.349Z</t>
+  </si>
+  <si>
+    <t>ACT-Bi32RrzI</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:27.657Z</t>
+  </si>
+  <si>
+    <t>ACT-JzCnGaHh</t>
+  </si>
+  <si>
+    <t>2026-09-04T07:32:27.730Z</t>
+  </si>
+  <si>
+    <t>ACT-hR36bHWu</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:21.433Z</t>
+  </si>
+  <si>
+    <t>ACT--GAM7Swl</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:21.485Z</t>
+  </si>
+  <si>
+    <t>ACT-1hI_bduP</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:22.439Z</t>
+  </si>
+  <si>
+    <t>ACT-Kqt5mb3z</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:22.476Z</t>
+  </si>
+  <si>
+    <t>ACT-lKAKkSmA</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:22.925Z</t>
+  </si>
+  <si>
+    <t>ACT-UOs767bJ</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:22.979Z</t>
+  </si>
+  <si>
+    <t>ACT-58pxnrSn</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:23.382Z</t>
+  </si>
+  <si>
+    <t>ACT-KQ809EXF</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:05:23.431Z</t>
+  </si>
+  <si>
+    <t>ACT-Qb14nG3j</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:17:42.735Z</t>
+  </si>
+  <si>
+    <t>ACT-YInSpchP</t>
   </si>
   <si>
     <t>CARD-8qeH-06h</t>
   </si>
   <si>
-    <t>Magazine</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:17:46.492Z</t>
-  </si>
-  <si>
-    <t>TODO</t>
+    <t>2026-09-04T08:17:46.512Z</t>
+  </si>
+  <si>
+    <t>ACT-BWJb7AzV</t>
   </si>
   <si>
     <t>CARD-qoYMpst5</t>
@@ -252,7 +468,10 @@
     <t>Agenda</t>
   </si>
   <si>
-    <t>2026-09-04T08:17:55.127Z</t>
+    <t>2026-09-04T08:17:55.144Z</t>
+  </si>
+  <si>
+    <t>ACT-vrv7YSWn</t>
   </si>
   <si>
     <t>CARD-fCoghZlP</t>
@@ -261,7 +480,10 @@
     <t>Hall Of Fame</t>
   </si>
   <si>
-    <t>2026-09-04T08:17:59.720Z</t>
+    <t>2026-09-04T08:17:59.733Z</t>
+  </si>
+  <si>
+    <t>ACT--rsNS8i-</t>
   </si>
   <si>
     <t>CARD-FIT2AkSf</t>
@@ -270,7 +492,10 @@
     <t>Skill Bridge</t>
   </si>
   <si>
-    <t>2026-09-04T08:18:04.669Z</t>
+    <t>2026-09-04T08:18:04.684Z</t>
+  </si>
+  <si>
+    <t>ACT-Np04NN4h</t>
   </si>
   <si>
     <t>CARD-_K0t2WZj</t>
@@ -279,237 +504,6 @@
     <t>SDEP (Student Developer Expo Prog)</t>
   </si>
   <si>
-    <t>2026-09-04T08:18:25.138Z</t>
-  </si>
-  <si>
-    <t>UpdateID</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>UpdateText</t>
-  </si>
-  <si>
-    <t>Progress</t>
-  </si>
-  <si>
-    <t>UPD-CYw0R8O_</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
-    <t>asdasd</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:21:01.458Z</t>
-  </si>
-  <si>
-    <t>UPD-7a2_iMz3</t>
-  </si>
-  <si>
-    <t>asdfsdaf</t>
-  </si>
-  <si>
-    <t>ActivityID</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>OldValue</t>
-  </si>
-  <si>
-    <t>NewValue</t>
-  </si>
-  <si>
-    <t>Timestamp</t>
-  </si>
-  <si>
-    <t>ACT-QCKcrs0o</t>
-  </si>
-  <si>
-    <t>CARD-wiVR66sH</t>
-  </si>
-  <si>
-    <t>Created card</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:23:53.517Z</t>
-  </si>
-  <si>
-    <t>ACT-6S9gKyUQ</t>
-  </si>
-  <si>
-    <t>CARD-y75Q3FLy</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:24:02.126Z</t>
-  </si>
-  <si>
-    <t>ACT-8Z7tZiIR</t>
-  </si>
-  <si>
-    <t>Moved card</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:04.946Z</t>
-  </si>
-  <si>
-    <t>ACT-unq1XO_V</t>
-  </si>
-  <si>
-    <t>Changed status</t>
-  </si>
-  <si>
-    <t>IN PROGRESS</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:05.842Z</t>
-  </si>
-  <si>
-    <t>ACT-zW2LshVp</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:05.903Z</t>
-  </si>
-  <si>
-    <t>ACT-G9JlU1GN</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:07.836Z</t>
-  </si>
-  <si>
-    <t>ACT-hP5mkb6C</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:15.843Z</t>
-  </si>
-  <si>
-    <t>ACT-yZk50wkS</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:15.910Z</t>
-  </si>
-  <si>
-    <t>ACT-kxPkqAQN</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:25.500Z</t>
-  </si>
-  <si>
-    <t>ACT-Nlwsh-Nr</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:25.561Z</t>
-  </si>
-  <si>
-    <t>ACT-IszKmJ30</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:27.279Z</t>
-  </si>
-  <si>
-    <t>ACT-egJr9HT1</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:27.349Z</t>
-  </si>
-  <si>
-    <t>ACT-Bi32RrzI</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:27.657Z</t>
-  </si>
-  <si>
-    <t>ACT-JzCnGaHh</t>
-  </si>
-  <si>
-    <t>2026-09-04T07:32:27.730Z</t>
-  </si>
-  <si>
-    <t>ACT-hR36bHWu</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:21.433Z</t>
-  </si>
-  <si>
-    <t>ACT--GAM7Swl</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:21.485Z</t>
-  </si>
-  <si>
-    <t>ACT-1hI_bduP</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:22.439Z</t>
-  </si>
-  <si>
-    <t>ACT-Kqt5mb3z</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:22.476Z</t>
-  </si>
-  <si>
-    <t>ACT-lKAKkSmA</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:22.925Z</t>
-  </si>
-  <si>
-    <t>ACT-UOs767bJ</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:22.979Z</t>
-  </si>
-  <si>
-    <t>ACT-58pxnrSn</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:23.382Z</t>
-  </si>
-  <si>
-    <t>ACT-KQ809EXF</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:05:23.431Z</t>
-  </si>
-  <si>
-    <t>ACT-Qb14nG3j</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:17:42.735Z</t>
-  </si>
-  <si>
-    <t>ACT-YInSpchP</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:17:46.512Z</t>
-  </si>
-  <si>
-    <t>ACT-BWJb7AzV</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:17:55.144Z</t>
-  </si>
-  <si>
-    <t>ACT-vrv7YSWn</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:17:59.733Z</t>
-  </si>
-  <si>
-    <t>ACT--rsNS8i-</t>
-  </si>
-  <si>
-    <t>2026-09-04T08:18:04.684Z</t>
-  </si>
-  <si>
-    <t>ACT-Np04NN4h</t>
-  </si>
-  <si>
     <t>2026-09-04T08:18:25.150Z</t>
   </si>
   <si>
@@ -574,6 +568,36 @@
   </si>
   <si>
     <t>2026-09-04T08:21:02.925Z</t>
+  </si>
+  <si>
+    <t>ACT-9t9EqJXs</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:23:31.591Z</t>
+  </si>
+  <si>
+    <t>ACT-E0OshWJk</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:23:34.132Z</t>
+  </si>
+  <si>
+    <t>ACT-S19MdhsD</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:23:34.179Z</t>
+  </si>
+  <si>
+    <t>ACT-LBUb_lwk</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:23:35.048Z</t>
+  </si>
+  <si>
+    <t>ACT-H1nOKnf8</t>
+  </si>
+  <si>
+    <t>2026-09-04T08:23:35.121Z</t>
   </si>
 </sst>
 </file>
@@ -1304,7 +1328,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="13" width="15" customWidth="1"/>
@@ -1368,10 +1392,10 @@
         <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="G2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
         <v>37</v>
@@ -1383,218 +1407,13 @@
         <v>7</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
         <v>72</v>
-      </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" t="s">
-        <v>74</v>
-      </c>
-      <c r="L3" t="s">
-        <v>74</v>
-      </c>
-      <c r="M3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4">
-        <v>3</v>
-      </c>
-      <c r="J4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" t="s">
-        <v>78</v>
-      </c>
-      <c r="L4" t="s">
-        <v>78</v>
-      </c>
-      <c r="M4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" t="s">
-        <v>68</v>
-      </c>
-      <c r="H5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" t="s">
-        <v>81</v>
-      </c>
-      <c r="L5" t="s">
-        <v>81</v>
-      </c>
-      <c r="M5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" t="s">
-        <v>68</v>
-      </c>
-      <c r="H6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I6">
-        <v>5</v>
-      </c>
-      <c r="J6" t="s">
-        <v>7</v>
-      </c>
-      <c r="K6" t="s">
-        <v>84</v>
-      </c>
-      <c r="L6" t="s">
-        <v>84</v>
-      </c>
-      <c r="M6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" t="s">
-        <v>86</v>
-      </c>
-      <c r="E7" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H7" t="s">
-        <v>37</v>
-      </c>
-      <c r="I7">
-        <v>6</v>
-      </c>
-      <c r="J7" t="s">
-        <v>7</v>
-      </c>
-      <c r="K7" t="s">
-        <v>87</v>
-      </c>
-      <c r="L7" t="s">
-        <v>87</v>
-      </c>
-      <c r="M7" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1613,7 +1432,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>60</v>
@@ -1622,16 +1441,16 @@
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>65</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -1642,19 +1461,19 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
         <v>37</v>
@@ -1663,27 +1482,27 @@
         <v>100</v>
       </c>
       <c r="H2" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="I2" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E3" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="F3" t="s">
         <v>37</v>
@@ -1692,10 +1511,10 @@
         <v>100</v>
       </c>
       <c r="H3" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="I3" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1706,7 +1525,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="15" customWidth="1"/>
@@ -1714,7 +1533,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>60</v>
@@ -1723,30 +1542,30 @@
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E2" t="s">
         <v>37</v>
@@ -1755,44 +1574,44 @@
         <v>67</v>
       </c>
       <c r="G2" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
         <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="G3" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="B4" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
         <v>51</v>
@@ -1801,67 +1620,67 @@
         <v>54</v>
       </c>
       <c r="G4" t="s">
-        <v>112</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="B5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
         <v>104</v>
       </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" t="s">
-        <v>114</v>
-      </c>
-      <c r="E5" t="s">
-        <v>75</v>
-      </c>
-      <c r="F5" t="s">
-        <v>115</v>
-      </c>
       <c r="G5" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B6" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
+        <v>103</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G6" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E7" t="s">
         <v>57</v>
@@ -1870,21 +1689,21 @@
         <v>51</v>
       </c>
       <c r="G7" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
         <v>51</v>
@@ -1893,44 +1712,44 @@
         <v>54</v>
       </c>
       <c r="G8" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" t="s">
         <v>104</v>
       </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" t="s">
-        <v>114</v>
-      </c>
-      <c r="E9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F9" t="s">
-        <v>115</v>
-      </c>
       <c r="G9" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="B10" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E10" t="s">
         <v>54</v>
@@ -1939,44 +1758,44 @@
         <v>57</v>
       </c>
       <c r="G10" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E11" t="s">
         <v>104</v>
       </c>
-      <c r="C11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" t="s">
-        <v>114</v>
-      </c>
-      <c r="E11" t="s">
-        <v>115</v>
-      </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G11" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E12" t="s">
         <v>57</v>
@@ -1985,44 +1804,44 @@
         <v>54</v>
       </c>
       <c r="G12" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="B13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" t="s">
         <v>104</v>
       </c>
-      <c r="C13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" t="s">
-        <v>114</v>
-      </c>
-      <c r="E13" t="s">
-        <v>71</v>
-      </c>
-      <c r="F13" t="s">
-        <v>115</v>
-      </c>
       <c r="G13" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
@@ -2031,44 +1850,44 @@
         <v>51</v>
       </c>
       <c r="G14" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" t="s">
+        <v>102</v>
+      </c>
+      <c r="E15" t="s">
         <v>104</v>
       </c>
-      <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" t="s">
-        <v>114</v>
-      </c>
-      <c r="E15" t="s">
-        <v>115</v>
-      </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G15" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="B16" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
         <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E16" t="s">
         <v>51</v>
@@ -2077,44 +1896,44 @@
         <v>54</v>
       </c>
       <c r="G16" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" t="s">
+        <v>102</v>
+      </c>
+      <c r="E17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" t="s">
         <v>104</v>
       </c>
-      <c r="C17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" t="s">
-        <v>114</v>
-      </c>
-      <c r="E17" t="s">
-        <v>71</v>
-      </c>
-      <c r="F17" t="s">
-        <v>115</v>
-      </c>
       <c r="G17" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="B18" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E18" t="s">
         <v>54</v>
@@ -2123,44 +1942,44 @@
         <v>57</v>
       </c>
       <c r="G18" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" t="s">
+        <v>102</v>
+      </c>
+      <c r="E19" t="s">
         <v>104</v>
       </c>
-      <c r="C19" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" t="s">
-        <v>114</v>
-      </c>
-      <c r="E19" t="s">
-        <v>115</v>
-      </c>
       <c r="F19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G19" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="B20" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E20" t="s">
         <v>57</v>
@@ -2169,44 +1988,44 @@
         <v>54</v>
       </c>
       <c r="G20" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="B21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" t="s">
+        <v>102</v>
+      </c>
+      <c r="E21" t="s">
+        <v>72</v>
+      </c>
+      <c r="F21" t="s">
         <v>104</v>
       </c>
-      <c r="C21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" t="s">
-        <v>114</v>
-      </c>
-      <c r="E21" t="s">
-        <v>71</v>
-      </c>
-      <c r="F21" t="s">
-        <v>115</v>
-      </c>
       <c r="G21" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="B22" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
         <v>7</v>
       </c>
       <c r="D22" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E22" t="s">
         <v>54</v>
@@ -2215,44 +2034,44 @@
         <v>51</v>
       </c>
       <c r="G22" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="B23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" t="s">
+        <v>102</v>
+      </c>
+      <c r="E23" t="s">
         <v>104</v>
       </c>
-      <c r="C23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" t="s">
-        <v>114</v>
-      </c>
-      <c r="E23" t="s">
-        <v>115</v>
-      </c>
       <c r="F23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G23" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C24" t="s">
         <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E24" t="s">
         <v>37</v>
@@ -2261,136 +2080,136 @@
         <v>67</v>
       </c>
       <c r="G24" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>145</v>
       </c>
       <c r="C25" t="s">
         <v>7</v>
       </c>
       <c r="D25" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E25" t="s">
         <v>37</v>
       </c>
       <c r="F25" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="G25" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>148</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E26" t="s">
         <v>37</v>
       </c>
       <c r="F26" t="s">
-        <v>77</v>
+        <v>149</v>
       </c>
       <c r="G26" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>152</v>
       </c>
       <c r="C27" t="s">
         <v>7</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E27" t="s">
         <v>37</v>
       </c>
       <c r="F27" t="s">
-        <v>80</v>
+        <v>153</v>
       </c>
       <c r="G27" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B28" t="s">
-        <v>82</v>
+        <v>156</v>
       </c>
       <c r="C28" t="s">
         <v>7</v>
       </c>
       <c r="D28" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E28" t="s">
         <v>37</v>
       </c>
       <c r="F28" t="s">
-        <v>83</v>
+        <v>157</v>
       </c>
       <c r="G28" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B29" t="s">
-        <v>85</v>
+        <v>160</v>
       </c>
       <c r="C29" t="s">
         <v>7</v>
       </c>
       <c r="D29" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="E29" t="s">
         <v>37</v>
       </c>
       <c r="F29" t="s">
-        <v>86</v>
+        <v>161</v>
       </c>
       <c r="G29" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C30" t="s">
         <v>7</v>
       </c>
       <c r="D30" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E30" t="s">
         <v>51</v>
@@ -2399,44 +2218,44 @@
         <v>54</v>
       </c>
       <c r="G30" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B31" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C31" t="s">
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E31" t="s">
-        <v>75</v>
+        <v>103</v>
       </c>
       <c r="F31" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G31" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C32" t="s">
         <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E32" t="s">
         <v>54</v>
@@ -2445,44 +2264,44 @@
         <v>57</v>
       </c>
       <c r="G32" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B33" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C33" t="s">
         <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E33" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="F33" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G33" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B34" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E34" t="s">
         <v>57</v>
@@ -2491,44 +2310,44 @@
         <v>54</v>
       </c>
       <c r="G34" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C35" t="s">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F35" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G35" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B36" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C36" t="s">
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E36" t="s">
         <v>54</v>
@@ -2537,76 +2356,191 @@
         <v>51</v>
       </c>
       <c r="G36" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B37" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C37" t="s">
         <v>7</v>
       </c>
       <c r="D37" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E37" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="F37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G37" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B38" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
       <c r="D38" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E38" t="s">
         <v>37</v>
       </c>
       <c r="F38" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="G38" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B39" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E39" t="s">
         <v>37</v>
       </c>
       <c r="F39" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="G39" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>184</v>
+      </c>
+      <c r="B40" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" t="s">
+        <v>92</v>
+      </c>
+      <c r="E40" t="s">
+        <v>37</v>
+      </c>
+      <c r="F40" t="s">
+        <v>67</v>
+      </c>
+      <c r="G40" t="s">
         <v>185</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>186</v>
+      </c>
+      <c r="B41" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" t="s">
+        <v>99</v>
+      </c>
+      <c r="E41" t="s">
+        <v>51</v>
+      </c>
+      <c r="F41" t="s">
+        <v>54</v>
+      </c>
+      <c r="G41" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>188</v>
+      </c>
+      <c r="B42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C42" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" t="s">
+        <v>102</v>
+      </c>
+      <c r="E42" t="s">
+        <v>103</v>
+      </c>
+      <c r="F42" t="s">
+        <v>104</v>
+      </c>
+      <c r="G42" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>190</v>
+      </c>
+      <c r="B43" t="s">
+        <v>66</v>
+      </c>
+      <c r="C43" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" t="s">
+        <v>99</v>
+      </c>
+      <c r="E43" t="s">
+        <v>54</v>
+      </c>
+      <c r="F43" t="s">
+        <v>51</v>
+      </c>
+      <c r="G43" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>192</v>
+      </c>
+      <c r="B44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" t="s">
+        <v>102</v>
+      </c>
+      <c r="E44" t="s">
+        <v>104</v>
+      </c>
+      <c r="F44" t="s">
+        <v>72</v>
+      </c>
+      <c r="G44" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>